<commit_message>
Update CT and IR templates for improved clarity and consistency
- Enhanced the CT scan template by updating header labels and measurement parameters for the operating potential section, ensuring better data representation.
- Refined the IR templates to standardize header formats and improve the organization of test sections, particularly for effective focal spot size and contrast resolution tests.
- Added new sample rows for specific tests to enhance clarity in expected results and improve overall reporting quality across templates.
</commit_message>
<xml_diff>
--- a/public/templates/CArm_Template.tmp.xlsx
+++ b/public/templates/CArm_Template.tmp.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:M55"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -997,25 +997,25 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>kVp</v>
+        <v>Time (s)</v>
       </c>
       <c r="B23" t="str">
-        <v>mAs</v>
+        <v>1.0</v>
       </c>
       <c r="C23" t="str">
-        <v>Output 1</v>
+        <v/>
       </c>
       <c r="D23" t="str">
-        <v>Output 2</v>
+        <v/>
       </c>
       <c r="E23" t="str">
-        <v>Output 3</v>
+        <v/>
       </c>
       <c r="F23" t="str">
-        <v>Output 4</v>
+        <v/>
       </c>
       <c r="G23" t="str">
-        <v>Output 5</v>
+        <v/>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -1029,25 +1029,25 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>80</v>
+        <v>kVp</v>
       </c>
       <c r="B24" t="str">
-        <v>100</v>
+        <v>mAs</v>
       </c>
       <c r="C24" t="str">
-        <v>10.5</v>
+        <v>Measured Output 1</v>
       </c>
       <c r="D24" t="str">
-        <v>10.4</v>
+        <v>Measured Output 2</v>
       </c>
       <c r="E24" t="str">
-        <v>10.6</v>
+        <v>Measured Output 3</v>
       </c>
       <c r="F24" t="str">
-        <v>10.5</v>
+        <v>Measured Output 4</v>
       </c>
       <c r="G24" t="str">
-        <v>10.5</v>
+        <v>Measured Output 5</v>
       </c>
       <c r="H24" t="str">
         <v/>
@@ -1061,25 +1061,25 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="B25" t="str">
         <v>100</v>
       </c>
       <c r="C25" t="str">
-        <v>12.1</v>
+        <v>10.5</v>
       </c>
       <c r="D25" t="str">
-        <v>12.0</v>
+        <v>10.4</v>
       </c>
       <c r="E25" t="str">
-        <v>12.2</v>
+        <v>10.6</v>
       </c>
       <c r="F25" t="str">
-        <v>12.1</v>
+        <v>10.5</v>
       </c>
       <c r="G25" t="str">
-        <v>12.0</v>
+        <v>10.5</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -1093,25 +1093,25 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Tolerance Operator</v>
+        <v>100</v>
       </c>
       <c r="B26" t="str">
-        <v>&lt;=</v>
+        <v>100</v>
       </c>
       <c r="C26" t="str">
-        <v/>
+        <v>12.1</v>
       </c>
       <c r="D26" t="str">
-        <v/>
+        <v>12.0</v>
       </c>
       <c r="E26" t="str">
-        <v/>
+        <v>12.2</v>
       </c>
       <c r="F26" t="str">
-        <v/>
+        <v>12.1</v>
       </c>
       <c r="G26" t="str">
-        <v/>
+        <v>12.0</v>
       </c>
       <c r="H26" t="str">
         <v/>
@@ -1125,138 +1125,147 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="B27" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
         <v>Tolerance Value (CoV)</v>
       </c>
-      <c r="B27" t="str">
+      <c r="B28" t="str">
         <v>0.02</v>
       </c>
-      <c r="C27" t="str">
-        <v/>
-      </c>
-      <c r="D27" t="str">
-        <v/>
-      </c>
-      <c r="E27" t="str">
-        <v/>
-      </c>
-      <c r="F27" t="str">
-        <v/>
-      </c>
-      <c r="G27" t="str">
-        <v/>
-      </c>
-      <c r="H27" t="str">
-        <v/>
-      </c>
-      <c r="I27" t="str">
-        <v/>
-      </c>
-      <c r="J27" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>TEST: LOW CONTRAST RESOLUTION</v>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Smallest Hole Size (mm)</v>
-      </c>
-      <c r="B30" t="str">
-        <v>Recommended Standard</v>
+        <v>TEST: LOW CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
+        <v>Smallest Hole Size (mm)</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Recommended Standard</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
         <v>1.0</v>
       </c>
-      <c r="B31" t="str">
+      <c r="B32" t="str">
         <v>&gt;= 1.0 mm</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>TEST: HIGH CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Measured Resolution (lp/mm)</v>
-      </c>
-      <c r="B34" t="str">
-        <v>Recommended Standard (lp/mm)</v>
+        <v>TEST: HIGH CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
+        <v>Measured Resolution (lp/mm)</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Recommended Standard (lp/mm)</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
         <v>2.0</v>
       </c>
-      <c r="B35" t="str">
+      <c r="B36" t="str">
         <v>&gt;= 2.0 lp/mm</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>TEST: EXPOSURE RATE AT TABLE TOP</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
-      </c>
-      <c r="B38" t="str">
-        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
-      </c>
-      <c r="C38" t="str">
-        <v>Min. Focus to Tabletop Distance</v>
-      </c>
-      <c r="D38" t="str">
-        <v>Distance (cm)</v>
-      </c>
-      <c r="E38" t="str">
-        <v>Applied kV</v>
-      </c>
-      <c r="F38" t="str">
-        <v>Applied mA</v>
-      </c>
-      <c r="G38" t="str">
-        <v>Exposure (cGy/Min)</v>
+        <v>TEST: EXPOSURE RATE AT TABLE TOP</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>10</v>
+        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
       </c>
       <c r="B39" t="str">
-        <v>5</v>
+        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
       </c>
       <c r="C39" t="str">
-        <v>30</v>
+        <v>Min. Focus to Tabletop Distance</v>
       </c>
       <c r="D39" t="str">
-        <v>100</v>
+        <v>Distance (cm)</v>
       </c>
       <c r="E39" t="str">
-        <v>80</v>
+        <v>Applied kV</v>
       </c>
       <c r="F39" t="str">
-        <v>100</v>
+        <v>Applied mA</v>
       </c>
       <c r="G39" t="str">
-        <v>0.5</v>
+        <v>Exposure (cGy/Min)</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="B40" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="C40" t="str">
-        <v/>
+        <v>30</v>
       </c>
       <c r="D40" t="str">
         <v>100</v>
@@ -1268,187 +1277,178 @@
         <v>100</v>
       </c>
       <c r="G40" t="str">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v/>
+      </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v/>
+      </c>
+      <c r="D41" t="str">
+        <v>100</v>
+      </c>
+      <c r="E41" t="str">
+        <v>80</v>
+      </c>
+      <c r="F41" t="str">
+        <v>100</v>
+      </c>
+      <c r="G41" t="str">
         <v>0.6</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>TEST: TUBE HOUSING LEAKAGE</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>FDD (cm)</v>
-      </c>
-      <c r="B43" t="str">
-        <v>kV</v>
-      </c>
-      <c r="C43" t="str">
-        <v>mA</v>
-      </c>
-      <c r="D43" t="str">
-        <v>Time (sec)</v>
-      </c>
-      <c r="E43" t="str">
-        <v>Workload (mA·min/week)</v>
-      </c>
-      <c r="F43" t="str">
-        <v>Tol Value</v>
-      </c>
-      <c r="G43" t="str">
-        <v>Tol Operator</v>
-      </c>
-      <c r="H43" t="str">
-        <v>Location</v>
-      </c>
-      <c r="I43" t="str">
-        <v>Front</v>
-      </c>
-      <c r="J43" t="str">
-        <v>Back</v>
-      </c>
-      <c r="K43" t="str">
-        <v>Left</v>
-      </c>
-      <c r="L43" t="str">
-        <v>Right</v>
-      </c>
-      <c r="M43" t="str">
-        <v>Top</v>
+        <v>TEST: TUBE HOUSING LEAKAGE</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>100</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B44" t="str">
-        <v>80</v>
+        <v>kV</v>
       </c>
       <c r="C44" t="str">
-        <v>100</v>
+        <v>mA</v>
       </c>
       <c r="D44" t="str">
-        <v>1</v>
+        <v>Time (sec)</v>
       </c>
       <c r="E44" t="str">
-        <v>1000</v>
+        <v>Workload (mA·min/week)</v>
       </c>
       <c r="F44" t="str">
-        <v>1.0</v>
+        <v>Tol Value</v>
       </c>
       <c r="G44" t="str">
-        <v>less than or equal to</v>
+        <v>Tol Operator</v>
       </c>
       <c r="H44" t="str">
-        <v>Tube</v>
+        <v>Location</v>
       </c>
       <c r="I44" t="str">
-        <v>0.05</v>
+        <v>Front</v>
       </c>
       <c r="J44" t="str">
-        <v>0.03</v>
+        <v>Back</v>
       </c>
       <c r="K44" t="str">
-        <v>0.06</v>
+        <v>Left</v>
       </c>
       <c r="L44" t="str">
-        <v>0.04</v>
+        <v>Right</v>
       </c>
       <c r="M44" t="str">
-        <v>0.02</v>
+        <v>Top</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="B45" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="C45" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="D45" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="E45" t="str">
-        <v/>
+        <v>1000</v>
       </c>
       <c r="F45" t="str">
-        <v/>
+        <v>1.0</v>
       </c>
       <c r="G45" t="str">
-        <v/>
+        <v>&lt;=</v>
       </c>
       <c r="H45" t="str">
+        <v>Tube</v>
+      </c>
+      <c r="I45" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="J45" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="K45" t="str">
+        <v>0.06</v>
+      </c>
+      <c r="L45" t="str">
+        <v>0.04</v>
+      </c>
+      <c r="M45" t="str">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v/>
+      </c>
+      <c r="B46" t="str">
+        <v/>
+      </c>
+      <c r="C46" t="str">
+        <v/>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+      <c r="G46" t="str">
+        <v/>
+      </c>
+      <c r="H46" t="str">
         <v>Collimator</v>
       </c>
-      <c r="I45" t="str">
+      <c r="I46" t="str">
         <v>0.02</v>
       </c>
-      <c r="J45" t="str">
+      <c r="J46" t="str">
         <v>0.02</v>
       </c>
-      <c r="K45" t="str">
+      <c r="K46" t="str">
         <v>0.03</v>
       </c>
-      <c r="L45" t="str">
+      <c r="L46" t="str">
         <v>0.01</v>
       </c>
-      <c r="M45" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>TEST: LINEARITY OF MA LOADING</v>
-      </c>
-      <c r="B47" t="str">
-        <v/>
-      </c>
-      <c r="C47" t="str">
-        <v/>
-      </c>
-      <c r="D47" t="str">
-        <v/>
-      </c>
-      <c r="E47" t="str">
-        <v/>
-      </c>
-      <c r="F47" t="str">
-        <v/>
-      </c>
-      <c r="G47" t="str">
-        <v/>
-      </c>
-      <c r="H47" t="str">
-        <v/>
-      </c>
-      <c r="I47" t="str">
-        <v/>
-      </c>
-      <c r="J47" t="str">
+      <c r="M46" t="str">
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>FDD (cm)</v>
+        <v>TEST: LINEARITY OF MA LOADING</v>
       </c>
       <c r="B48" t="str">
-        <v>100</v>
+        <v/>
       </c>
       <c r="C48" t="str">
-        <v>kV</v>
+        <v/>
       </c>
       <c r="D48" t="str">
-        <v>80</v>
+        <v/>
       </c>
       <c r="E48" t="str">
-        <v>Time (s)</v>
+        <v/>
       </c>
       <c r="F48" t="str">
-        <v>0.1</v>
+        <v/>
       </c>
       <c r="G48" t="str">
         <v/>
@@ -1465,22 +1465,22 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>mA Applied</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B49" t="str">
-        <v>Measured Output 1</v>
+        <v>100</v>
       </c>
       <c r="C49" t="str">
-        <v>Measured Output 2</v>
+        <v>kV</v>
       </c>
       <c r="D49" t="str">
-        <v>Measured Output 3</v>
+        <v>80</v>
       </c>
       <c r="E49" t="str">
-        <v/>
+        <v>Time (s)</v>
       </c>
       <c r="F49" t="str">
-        <v/>
+        <v>0.1</v>
       </c>
       <c r="G49" t="str">
         <v/>
@@ -1497,16 +1497,16 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>50</v>
+        <v>mA Applied</v>
       </c>
       <c r="B50" t="str">
-        <v>0.10</v>
+        <v>Measured Output 1</v>
       </c>
       <c r="C50" t="str">
-        <v>0.11</v>
+        <v>Measured Output 2</v>
       </c>
       <c r="D50" t="str">
-        <v>0.09</v>
+        <v>Measured Output 3</v>
       </c>
       <c r="E50" t="str">
         <v/>
@@ -1529,16 +1529,16 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>0.20</v>
+        <v>0.10</v>
       </c>
       <c r="C51" t="str">
-        <v>0.21</v>
+        <v>0.11</v>
       </c>
       <c r="D51" t="str">
-        <v>0.19</v>
+        <v>0.09</v>
       </c>
       <c r="E51" t="str">
         <v/>
@@ -1561,16 +1561,16 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="B52" t="str">
-        <v>0.40</v>
+        <v>0.20</v>
       </c>
       <c r="C52" t="str">
-        <v>0.41</v>
+        <v>0.21</v>
       </c>
       <c r="D52" t="str">
-        <v>0.39</v>
+        <v>0.19</v>
       </c>
       <c r="E52" t="str">
         <v/>
@@ -1593,16 +1593,16 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Tolerance Operator</v>
+        <v>200</v>
       </c>
       <c r="B53" t="str">
-        <v>&lt;=</v>
+        <v>0.40</v>
       </c>
       <c r="C53" t="str">
-        <v/>
+        <v>0.41</v>
       </c>
       <c r="D53" t="str">
-        <v/>
+        <v>0.39</v>
       </c>
       <c r="E53" t="str">
         <v/>
@@ -1625,46 +1625,78 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="B54" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="C54" t="str">
+        <v/>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
+      <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
         <v>Tolerance Value (CoL)</v>
       </c>
-      <c r="B54" t="str">
+      <c r="B55" t="str">
         <v>0.1</v>
       </c>
-      <c r="C54" t="str">
-        <v/>
-      </c>
-      <c r="D54" t="str">
-        <v/>
-      </c>
-      <c r="E54" t="str">
-        <v/>
-      </c>
-      <c r="F54" t="str">
-        <v/>
-      </c>
-      <c r="G54" t="str">
-        <v/>
-      </c>
-      <c r="H54" t="str">
-        <v/>
-      </c>
-      <c r="I54" t="str">
-        <v/>
-      </c>
-      <c r="J54" t="str">
+      <c r="C55" t="str">
+        <v/>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
+      <c r="H55" t="str">
+        <v/>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M55"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M50"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -2166,25 +2198,25 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>kVp</v>
+        <v>Time (s)</v>
       </c>
       <c r="B17" t="str">
-        <v>mAs</v>
+        <v>1.0</v>
       </c>
       <c r="C17" t="str">
-        <v>Output 1</v>
+        <v/>
       </c>
       <c r="D17" t="str">
-        <v>Output 2</v>
+        <v/>
       </c>
       <c r="E17" t="str">
-        <v>Output 3</v>
+        <v/>
       </c>
       <c r="F17" t="str">
-        <v>Output 4</v>
+        <v/>
       </c>
       <c r="G17" t="str">
-        <v>Output 5</v>
+        <v/>
       </c>
       <c r="H17" t="str">
         <v/>
@@ -2198,25 +2230,25 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>80</v>
+        <v>kVp</v>
       </c>
       <c r="B18" t="str">
-        <v>100</v>
+        <v>mAs</v>
       </c>
       <c r="C18" t="str">
-        <v>10.5</v>
+        <v>Measured Output 1</v>
       </c>
       <c r="D18" t="str">
-        <v>10.4</v>
+        <v>Measured Output 2</v>
       </c>
       <c r="E18" t="str">
-        <v>10.6</v>
+        <v>Measured Output 3</v>
       </c>
       <c r="F18" t="str">
-        <v>10.5</v>
+        <v>Measured Output 4</v>
       </c>
       <c r="G18" t="str">
-        <v>10.5</v>
+        <v>Measured Output 5</v>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -2230,25 +2262,25 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="B19" t="str">
         <v>100</v>
       </c>
       <c r="C19" t="str">
-        <v>12.1</v>
+        <v>10.5</v>
       </c>
       <c r="D19" t="str">
-        <v>12.0</v>
+        <v>10.4</v>
       </c>
       <c r="E19" t="str">
-        <v>12.2</v>
+        <v>10.6</v>
       </c>
       <c r="F19" t="str">
-        <v>12.1</v>
+        <v>10.5</v>
       </c>
       <c r="G19" t="str">
-        <v>12.0</v>
+        <v>10.5</v>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -2262,25 +2294,25 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Tolerance Operator</v>
+        <v>100</v>
       </c>
       <c r="B20" t="str">
-        <v>&lt;=</v>
+        <v>100</v>
       </c>
       <c r="C20" t="str">
-        <v/>
+        <v>12.1</v>
       </c>
       <c r="D20" t="str">
-        <v/>
+        <v>12.0</v>
       </c>
       <c r="E20" t="str">
-        <v/>
+        <v>12.2</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>12.1</v>
       </c>
       <c r="G20" t="str">
-        <v/>
+        <v>12.0</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -2294,138 +2326,147 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="B21" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
         <v>Tolerance Value (CoV)</v>
       </c>
-      <c r="B21" t="str">
+      <c r="B22" t="str">
         <v>0.02</v>
       </c>
-      <c r="C21" t="str">
-        <v/>
-      </c>
-      <c r="D21" t="str">
-        <v/>
-      </c>
-      <c r="E21" t="str">
-        <v/>
-      </c>
-      <c r="F21" t="str">
-        <v/>
-      </c>
-      <c r="G21" t="str">
-        <v/>
-      </c>
-      <c r="H21" t="str">
-        <v/>
-      </c>
-      <c r="I21" t="str">
-        <v/>
-      </c>
-      <c r="J21" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>TEST: LOW CONTRAST RESOLUTION</v>
+      <c r="C22" t="str">
+        <v/>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Smallest Hole Size (mm)</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Recommended Standard</v>
+        <v>TEST: LOW CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
+        <v>Smallest Hole Size (mm)</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Recommended Standard</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
         <v>1.0</v>
       </c>
-      <c r="B25" t="str">
+      <c r="B26" t="str">
         <v>&gt;= 1.0 mm</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>TEST: HIGH CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Measured Resolution (lp/mm)</v>
-      </c>
-      <c r="B28" t="str">
-        <v>Recommended Standard (lp/mm)</v>
+        <v>TEST: HIGH CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
+        <v>Measured Resolution (lp/mm)</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Recommended Standard (lp/mm)</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
         <v>2.0</v>
       </c>
-      <c r="B29" t="str">
+      <c r="B30" t="str">
         <v>&gt;= 2.0 lp/mm</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>TEST: EXPOSURE RATE AT TABLE TOP</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
-      </c>
-      <c r="B32" t="str">
-        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
-      </c>
-      <c r="C32" t="str">
-        <v>Min. Focus to Tabletop Distance</v>
-      </c>
-      <c r="D32" t="str">
-        <v>Distance (cm)</v>
-      </c>
-      <c r="E32" t="str">
-        <v>Applied kV</v>
-      </c>
-      <c r="F32" t="str">
-        <v>Applied mA</v>
-      </c>
-      <c r="G32" t="str">
-        <v>Exposure (cGy/Min)</v>
+        <v>TEST: EXPOSURE RATE AT TABLE TOP</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>10</v>
+        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
       </c>
       <c r="B33" t="str">
-        <v>5</v>
+        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
       </c>
       <c r="C33" t="str">
-        <v>30</v>
+        <v>Min. Focus to Tabletop Distance</v>
       </c>
       <c r="D33" t="str">
-        <v>100</v>
+        <v>Distance (cm)</v>
       </c>
       <c r="E33" t="str">
-        <v>80</v>
+        <v>Applied kV</v>
       </c>
       <c r="F33" t="str">
-        <v>100</v>
+        <v>Applied mA</v>
       </c>
       <c r="G33" t="str">
-        <v>0.5</v>
+        <v>Exposure (cGy/Min)</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="B34" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="C34" t="str">
-        <v/>
+        <v>30</v>
       </c>
       <c r="D34" t="str">
         <v>100</v>
@@ -2437,181 +2478,172 @@
         <v>100</v>
       </c>
       <c r="G34" t="str">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v>100</v>
+      </c>
+      <c r="E35" t="str">
+        <v>80</v>
+      </c>
+      <c r="F35" t="str">
+        <v>100</v>
+      </c>
+      <c r="G35" t="str">
         <v>0.6</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>TEST: TUBE HOUSING LEAKAGE</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>FDD (cm)</v>
-      </c>
-      <c r="B37" t="str">
-        <v>kV</v>
-      </c>
-      <c r="C37" t="str">
-        <v>mA</v>
-      </c>
-      <c r="D37" t="str">
-        <v>Time (sec)</v>
-      </c>
-      <c r="E37" t="str">
-        <v>Workload (mA·min/week)</v>
-      </c>
-      <c r="F37" t="str">
-        <v>Tol Value</v>
-      </c>
-      <c r="G37" t="str">
-        <v>Tol Operator</v>
-      </c>
-      <c r="H37" t="str">
-        <v>Location</v>
-      </c>
-      <c r="I37" t="str">
-        <v>Front</v>
-      </c>
-      <c r="J37" t="str">
-        <v>Back</v>
-      </c>
-      <c r="K37" t="str">
-        <v>Left</v>
-      </c>
-      <c r="L37" t="str">
-        <v>Right</v>
-      </c>
-      <c r="M37" t="str">
-        <v>Top</v>
+        <v>TEST: TUBE HOUSING LEAKAGE</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>100</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B38" t="str">
-        <v>80</v>
+        <v>kV</v>
       </c>
       <c r="C38" t="str">
-        <v>100</v>
+        <v>mA</v>
       </c>
       <c r="D38" t="str">
-        <v>1</v>
+        <v>Time (sec)</v>
       </c>
       <c r="E38" t="str">
-        <v>1000</v>
+        <v>Workload (mA·min/week)</v>
       </c>
       <c r="F38" t="str">
-        <v>1.0</v>
+        <v>Tol Value</v>
       </c>
       <c r="G38" t="str">
-        <v>less than or equal to</v>
+        <v>Tol Operator</v>
       </c>
       <c r="H38" t="str">
-        <v>Tube</v>
+        <v>Location</v>
       </c>
       <c r="I38" t="str">
-        <v>0.05</v>
+        <v>Front</v>
       </c>
       <c r="J38" t="str">
-        <v>0.03</v>
+        <v>Back</v>
       </c>
       <c r="K38" t="str">
-        <v>0.06</v>
+        <v>Left</v>
       </c>
       <c r="L38" t="str">
-        <v>0.04</v>
+        <v>Right</v>
       </c>
       <c r="M38" t="str">
-        <v>0.02</v>
+        <v>Top</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="B39" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="C39" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="D39" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="E39" t="str">
-        <v/>
+        <v>1000</v>
       </c>
       <c r="F39" t="str">
-        <v/>
+        <v>1.0</v>
       </c>
       <c r="G39" t="str">
-        <v/>
+        <v>&lt;=</v>
       </c>
       <c r="H39" t="str">
+        <v>Tube</v>
+      </c>
+      <c r="I39" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="J39" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="K39" t="str">
+        <v>0.06</v>
+      </c>
+      <c r="L39" t="str">
+        <v>0.04</v>
+      </c>
+      <c r="M39" t="str">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v/>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
         <v>Collimator</v>
       </c>
-      <c r="I39" t="str">
+      <c r="I40" t="str">
         <v>0.02</v>
       </c>
-      <c r="J39" t="str">
+      <c r="J40" t="str">
         <v>0.02</v>
       </c>
-      <c r="K39" t="str">
+      <c r="K40" t="str">
         <v>0.03</v>
       </c>
-      <c r="L39" t="str">
+      <c r="L40" t="str">
         <v>0.01</v>
       </c>
-      <c r="M39" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>TEST: LINEARITY OF MAS LOADING</v>
-      </c>
-      <c r="B41" t="str">
-        <v/>
-      </c>
-      <c r="C41" t="str">
-        <v/>
-      </c>
-      <c r="D41" t="str">
-        <v/>
-      </c>
-      <c r="E41" t="str">
-        <v/>
-      </c>
-      <c r="F41" t="str">
-        <v/>
-      </c>
-      <c r="G41" t="str">
-        <v/>
-      </c>
-      <c r="H41" t="str">
-        <v/>
-      </c>
-      <c r="I41" t="str">
-        <v/>
-      </c>
-      <c r="J41" t="str">
+      <c r="M40" t="str">
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>FDD (cm)</v>
+        <v>TEST: LINEARITY OF MAS LOADING</v>
       </c>
       <c r="B42" t="str">
-        <v>100</v>
+        <v/>
       </c>
       <c r="C42" t="str">
-        <v>kV</v>
+        <v/>
       </c>
       <c r="D42" t="str">
-        <v>80</v>
+        <v/>
       </c>
       <c r="E42" t="str">
         <v/>
@@ -2634,16 +2666,16 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>mAs Range</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B43" t="str">
-        <v>Measured Output 1</v>
+        <v>100</v>
       </c>
       <c r="C43" t="str">
-        <v>Measured Output 2</v>
+        <v>kV</v>
       </c>
       <c r="D43" t="str">
-        <v>Measured Output 3</v>
+        <v>80</v>
       </c>
       <c r="E43" t="str">
         <v/>
@@ -2666,16 +2698,16 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>5 - 10</v>
+        <v>mAs</v>
       </c>
       <c r="B44" t="str">
-        <v>0.50</v>
+        <v>Measured Output 1</v>
       </c>
       <c r="C44" t="str">
-        <v>0.51</v>
+        <v>Measured Output 2</v>
       </c>
       <c r="D44" t="str">
-        <v>0.49</v>
+        <v>Measured Output 3</v>
       </c>
       <c r="E44" t="str">
         <v/>
@@ -2698,16 +2730,16 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>10 - 20</v>
+        <v>5</v>
       </c>
       <c r="B45" t="str">
-        <v>1.00</v>
+        <v>0.50</v>
       </c>
       <c r="C45" t="str">
-        <v>1.01</v>
+        <v>0.51</v>
       </c>
       <c r="D45" t="str">
-        <v>0.99</v>
+        <v>0.49</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -2730,16 +2762,16 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>20 - 50</v>
+        <v>10</v>
       </c>
       <c r="B46" t="str">
-        <v>2.50</v>
+        <v>1.00</v>
       </c>
       <c r="C46" t="str">
-        <v>2.51</v>
+        <v>1.01</v>
       </c>
       <c r="D46" t="str">
-        <v>2.49</v>
+        <v>0.99</v>
       </c>
       <c r="E46" t="str">
         <v/>
@@ -2762,16 +2794,16 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>50 - 100</v>
+        <v>20</v>
       </c>
       <c r="B47" t="str">
-        <v>5.00</v>
+        <v>2.50</v>
       </c>
       <c r="C47" t="str">
-        <v>5.01</v>
+        <v>2.51</v>
       </c>
       <c r="D47" t="str">
-        <v>4.99</v>
+        <v>2.49</v>
       </c>
       <c r="E47" t="str">
         <v/>
@@ -2794,16 +2826,16 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Tolerance Operator</v>
+        <v>50</v>
       </c>
       <c r="B48" t="str">
-        <v>&lt;=</v>
+        <v>5.00</v>
       </c>
       <c r="C48" t="str">
-        <v/>
+        <v>5.01</v>
       </c>
       <c r="D48" t="str">
-        <v/>
+        <v>4.99</v>
       </c>
       <c r="E48" t="str">
         <v/>
@@ -2826,39 +2858,71 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="B49" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="C49" t="str">
+        <v/>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
         <v>Tolerance Value (CoL)</v>
       </c>
-      <c r="B49" t="str">
+      <c r="B50" t="str">
         <v>0.1</v>
       </c>
-      <c r="C49" t="str">
-        <v/>
-      </c>
-      <c r="D49" t="str">
-        <v/>
-      </c>
-      <c r="E49" t="str">
-        <v/>
-      </c>
-      <c r="F49" t="str">
-        <v/>
-      </c>
-      <c r="G49" t="str">
-        <v/>
-      </c>
-      <c r="H49" t="str">
-        <v/>
-      </c>
-      <c r="I49" t="str">
-        <v/>
-      </c>
-      <c r="J49" t="str">
+      <c r="C50" t="str">
+        <v/>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+      <c r="G50" t="str">
+        <v/>
+      </c>
+      <c r="H50" t="str">
+        <v/>
+      </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M50"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update templates for CArm and Dental tests to standardize terminology and improve data structure
- Changed 'mA Station' to 'mAs Station' in various test data templates for consistency.
- Updated tolerance signs and values in the Dental CBCT and OPG templates to enhance clarity.
- Refined test data formats across multiple templates to ensure uniformity in reporting and usability.
</commit_message>
<xml_diff>
--- a/public/templates/CArm_Template.tmp.xlsx
+++ b/public/templates/CArm_Template.tmp.xlsx
@@ -677,7 +677,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>mA Station 1</v>
+        <v>mAs Station 1</v>
       </c>
       <c r="B12" t="str">
         <v>50</v>
@@ -709,7 +709,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>mA Station 2</v>
+        <v>mAs Station 2</v>
       </c>
       <c r="B13" t="str">
         <v>100</v>
@@ -741,7 +741,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>mA Station 3</v>
+        <v>mAs Station 3</v>
       </c>
       <c r="B14" t="str">
         <v>200</v>
@@ -1256,6 +1256,9 @@
       <c r="G39" t="str">
         <v>Exposure (cGy/Min)</v>
       </c>
+      <c r="H39" t="str">
+        <v>Mode</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1279,6 +1282,9 @@
       <c r="G40" t="str">
         <v>0.5</v>
       </c>
+      <c r="H40" t="str">
+        <v>AEC Mode</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1301,6 +1307,9 @@
       </c>
       <c r="G41" t="str">
         <v>0.6</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Manual Mode</v>
       </c>
     </row>
     <row r="43">
@@ -1878,7 +1887,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>mA Station 1</v>
+        <v>mAs Station 1</v>
       </c>
       <c r="B6" t="str">
         <v>50</v>
@@ -1910,7 +1919,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>mA Station 2</v>
+        <v>mAs Station 2</v>
       </c>
       <c r="B7" t="str">
         <v>100</v>
@@ -1942,7 +1951,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>mA Station 3</v>
+        <v>mAs Station 3</v>
       </c>
       <c r="B8" t="str">
         <v>200</v>
@@ -2457,6 +2466,9 @@
       <c r="G33" t="str">
         <v>Exposure (cGy/Min)</v>
       </c>
+      <c r="H33" t="str">
+        <v>Mode</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -2480,6 +2492,9 @@
       <c r="G34" t="str">
         <v>0.5</v>
       </c>
+      <c r="H34" t="str">
+        <v>AEC Mode</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2502,6 +2517,9 @@
       </c>
       <c r="G35" t="str">
         <v>0.6</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Manual Mode</v>
       </c>
     </row>
     <row r="37">

</xml_diff>